<commit_message>
new ui, excel output
</commit_message>
<xml_diff>
--- a/dist/time_tracker_2026-04.xlsx
+++ b/dist/time_tracker_2026-04.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Time Entries'!$A$1:$J$57</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Time Entries'!$A$1:$J$58</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J57"/>
+  <dimension ref="A1:J58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2879,27 +2879,27 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>2026-04-15T12:00:01.578900</t>
+          <t>2026-04-15T14:34:45.121513</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>2026-04-15T12:00:13.633823</t>
+          <t>2026-04-15T14:36:37.359775</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t>0.02</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Black-Jack</t>
+          <t>FERRARI-IT-24-01-10</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>104180001560</t>
+          <t>S-2103578413</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -2907,13 +2907,21 @@
           <t>114000</t>
         </is>
       </c>
-      <c r="H55" s="3" t="inlineStr"/>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>0130</t>
+        </is>
+      </c>
       <c r="I55" t="inlineStr">
         <is>
           <t>D330000</t>
         </is>
       </c>
-      <c r="J55" s="3" t="inlineStr"/>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>longtime run</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
@@ -3011,8 +3019,54 @@
         </is>
       </c>
     </row>
+    <row r="58">
+      <c r="A58" s="2" t="n">
+        <v>46127</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>2026-04-15T12:00:01</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>2026-04-15T12:00:13</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Black-Jack</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>104180001560</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>114000</t>
+        </is>
+      </c>
+      <c r="H58" s="3" t="inlineStr"/>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>D330000</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>ttt</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J57"/>
+  <autoFilter ref="A1:J58"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3045,7 +3099,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>20.26</v>
+        <v>20.28</v>
       </c>
     </row>
     <row r="3">
@@ -3055,7 +3109,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="4">
@@ -3066,7 +3120,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-04-15 12:08:36</t>
+          <t>2026-04-15 14:36:49</t>
         </is>
       </c>
     </row>

</xml_diff>